<commit_message>
fix: rebuild launch-skus.xlsx with variant-level data from Medusa
15 products, 30 variants with actual SKU codes (CL-XXX-XXXX) and
prices pulled from production Medusa. Each variant is its own row.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ops/launch-skus.xlsx
+++ b/docs/ops/launch-skus.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,28 @@
     <font>
       <name val="Arial"/>
       <color rgb="00111111"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00111111"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00111111"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="007090AB"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007090AB"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -83,17 +105,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,13 +495,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,15 +514,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Variant</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Variants</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Price (USD)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
@@ -494,239 +542,311 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>BPC-157</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>5mg, 10mg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>CL-BPC-0005</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>$1</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Repair</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>GHK-Cu</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>50mg, 100mg</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Repair</t>
-        </is>
-      </c>
+      <c r="B3" s="6" t="inlineStr"/>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>CL-BPC-0010</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>$2</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>GLP1-S</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TB-500</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>10mg, 20mg, 30mg</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Metabolic</t>
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>CL-TB5-0005</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>$1</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Repair</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>GLP2-T</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>10mg, 20mg, 30mg</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Metabolic</t>
-        </is>
-      </c>
+      <c r="B5" s="6" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>CL-TB5-0010</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>$2</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>GLP3-R</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>GHK-Cu</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>10mg, 20mg, 30mg</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Metabolic</t>
+          <t>50mg</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>CL-GHK-0050</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Repair</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Ipamorelin</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>5mg, 10mg</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>GH Axis</t>
-        </is>
-      </c>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>100mg</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>CL-GHK-0100</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>MOTS-c</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Wolverine</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>10mg, 40mg</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Longevity</t>
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>CL-WLV-0005</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>$199</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Repair</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>SS-31</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>10mg, 50mg</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Longevity</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>CL-WLV-0010</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>$349</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>TB-500</t>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>GLP1-S</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>5mg, 10mg</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Repair</t>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>CL-GL1-0010</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>$159</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Metabolic</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Tesamorelin</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>10mg, 20mg</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>GH Axis</t>
-        </is>
-      </c>
+      <c r="B11" s="6" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>20mg</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>CL-GL1-0020</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>$289</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Wolverine</t>
-        </is>
-      </c>
+      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>5mg, 10mg</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Repair</t>
-        </is>
-      </c>
+          <t>30mg</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>CL-GL1-0030</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>$399</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Glow</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>70mg</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Adjacent</t>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>GLP2-T</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>CL-GL2-0010</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>$159</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Metabolic</t>
         </is>
       </c>
     </row>
@@ -734,59 +854,479 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Klow</t>
-        </is>
-      </c>
+      <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>80mg</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Adjacent</t>
-        </is>
-      </c>
+          <t>20mg</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>CL-GL2-0020</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>$289</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Melanotan 2</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Adjacent</t>
-        </is>
-      </c>
+      <c r="B15" s="6" t="inlineStr"/>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>30mg</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>CL-GL2-0030</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>$399</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>GLP3-R</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>CL-GL3-0010</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>$179</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Metabolic</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>20mg</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>CL-GL3-0020</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>$329</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>30mg</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>CL-GL3-0030</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>$449</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Ipamorelin</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>CL-IPM-0005</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>$35</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>GH Axis</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>CL-IPM-0010</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Tesamorelin</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>CL-TES-0010</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>$179</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>GH Axis</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>20mg</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>CL-TES-0020</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>$329</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>MOTS-c</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>CL-MOT-0010</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>$3</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Longevity</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>40mg</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>CL-MOT-0040</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>$9</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>SS-31</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>CL-SS3-0010</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>$129</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Longevity</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>50mg</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>CL-SS3-0050</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>$549</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>GLOW</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>70mg</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>CL-GLW-0070</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>$1</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>KLOW</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>80mg</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>CL-KLW-0080</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>$1</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Melanotan 2</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>CL-MT2-0010</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Bac Water</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>3mL, 10mL</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>3mL</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>CL-BAC-0003</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr"/>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>10mL</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>CL-BAC-0010</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>15 products, 30 variants</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add QR marketing attribution system design spec
Design for @calilean/plugin-qr-marketing — QR codes on peptide pens
and marketing materials with Segment attribution tracking, admin UI
for campaign management, and storefront UTM cookie persistence.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ops/launch-skus.xlsx
+++ b/docs/ops/launch-skus.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,37 +26,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <color rgb="00111111"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00111111"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <color rgb="00111111"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <color rgb="007090AB"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="007090AB"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -68,14 +43,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00111111"/>
-        <bgColor rgb="00111111"/>
+        <fgColor rgb="002D3748"/>
+        <bgColor rgb="002D3748"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F0"/>
-        <bgColor rgb="00F0F0F0"/>
+        <fgColor rgb="00F7FAFC"/>
+        <bgColor rgb="00F7FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,48 +63,24 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00E5E5E5"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E5E5E5"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E5E5E5"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E5E5E5"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,15 +446,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,7 +493,7 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>BPC-157</t>
         </is>
@@ -552,14 +503,14 @@
           <t>5mg</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CL-BPC-0005</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>$1</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -569,32 +520,32 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>CL-BPC-0010</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>$2</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>$59.99</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>TB-500</t>
         </is>
@@ -604,14 +555,14 @@
           <t>5mg</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>CL-TB5-0005</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>$1</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>$39.99</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -621,32 +572,32 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>CL-TB5-0010</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>$2</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>$69.99</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>GHK-Cu</t>
         </is>
@@ -656,14 +607,14 @@
           <t>50mg</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>CL-GHK-0050</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>$39.99</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -673,32 +624,32 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>100mg</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>CL-GHK-0100</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>$69.99</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Wolverine</t>
         </is>
@@ -708,14 +659,14 @@
           <t>5mg</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>CL-WLV-0005</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>$199</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>$69.99</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -725,32 +676,32 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr"/>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>CL-WLV-0010</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>$349</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>$99.99</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>GLP1-S</t>
         </is>
@@ -760,14 +711,14 @@
           <t>10mg</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>CL-GL1-0010</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>$159</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>$69.99</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -777,74 +728,74 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="inlineStr"/>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>CL-GL1-0020</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>$289</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>$119.99</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
           <t>30mg</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>CL-GL1-0030</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>$399</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>$159.99</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>GLP2-T</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>CL-GL2-0010</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>$159</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>$79.99</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Metabolic</t>
         </is>
@@ -854,51 +805,51 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>CL-GL2-0020</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>$289</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>$139.99</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="inlineStr"/>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>30mg</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>CL-GL2-0030</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>$399</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>$189.99</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>GLP3-R</t>
         </is>
@@ -908,14 +859,14 @@
           <t>10mg</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>CL-GL3-0010</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>$179</t>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>$79.99</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -925,74 +876,74 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="inlineStr"/>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>CL-GL3-0020</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>$329</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr"/>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>$149.99</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
           <t>30mg</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>CL-GL3-0030</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>$449</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>$219.99</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Ipamorelin</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>CL-IPM-0005</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>$35</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>$34.99</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>GH Axis</t>
         </is>
@@ -1002,49 +953,49 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>CL-IPM-0010</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>$54.99</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Tesamorelin</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>CL-TES-0010</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>$179</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>$69.99</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>GH Axis</t>
         </is>
@@ -1054,49 +1005,49 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>CL-TES-0020</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>$329</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>$119.99</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>MOTS-c</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>CL-MOT-0010</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>$3</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>$44.99</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Longevity</t>
         </is>
@@ -1106,49 +1057,49 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>40mg</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>CL-MOT-0040</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>$9</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>$109.99</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>SS-31</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>CL-SS3-0010</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>$129</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>$59.99</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Longevity</t>
         </is>
@@ -1158,49 +1109,49 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>50mg</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>CL-SS3-0050</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>$549</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>$199.99</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>GLOW</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>70mg</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>CL-GLW-0070</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>$1</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>$89.99</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Specialty</t>
         </is>
@@ -1210,7 +1161,7 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>KLOW</t>
         </is>
@@ -1220,14 +1171,14 @@
           <t>80mg</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>CL-KLW-0080</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>$1</t>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>$119.99</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1237,30 +1188,30 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n">
+      <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Melanotan 2</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>10mg</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>CL-MT2-0010</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>$34.99</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Specialty</t>
         </is>
@@ -1270,7 +1221,7 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Bac Water</t>
         </is>
@@ -1280,14 +1231,14 @@
           <t>3mL</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>CL-BAC-0003</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>$10</t>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>$9.99</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1297,38 +1248,42 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="6" t="inlineStr"/>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>10mL</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>CL-BAC-0010</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>$14.99</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>15 products, 30 variants</t>
         </is>
       </c>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>